<commit_message>
version final para entrega formal
</commit_message>
<xml_diff>
--- a/gantt/Gantt_CasaMonarca_MA2006B.xlsx
+++ b/gantt/Gantt_CasaMonarca_MA2006B.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marielalvarez/2026/6toSem/reto_cripto_final/Casa-Monarca-Criptografia/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marielalvarez/2026/6toSem/reto_cripto_final/Casa-Monarca-Criptografia/gantt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312A792E-EC3E-D546-837B-981E3E130261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70873041-25A6-774E-B8C5-3FBA24453146}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="920" yWindow="-18540" windowWidth="29400" windowHeight="18480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="920" yWindow="-18540" windowWidth="29400" windowHeight="18480" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Gantt" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="921" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="451">
   <si>
     <t>CASA MONARCA CRIPTOGRAFÍA — Cronograma de Proyecto MA2006B · 2026</t>
   </si>
@@ -1378,6 +1378,9 @@
   </si>
   <si>
     <t>Brisma, Emiliano</t>
+  </si>
+  <si>
+    <t>Correcciones finales</t>
   </si>
 </sst>
 </file>
@@ -1848,13 +1851,6 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="19" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1863,6 +1859,13 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2166,7 +2169,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X91"/>
+  <dimension ref="A1:X92"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -2181,32 +2184,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
-      <c r="O1" s="78"/>
-      <c r="P1" s="78"/>
-      <c r="Q1" s="78"/>
-      <c r="R1" s="78"/>
-      <c r="S1" s="78"/>
-      <c r="T1" s="78"/>
-      <c r="U1" s="78"/>
-      <c r="V1" s="78"/>
-      <c r="W1" s="78"/>
-      <c r="X1" s="78"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
+      <c r="E1" s="81"/>
+      <c r="F1" s="81"/>
+      <c r="G1" s="81"/>
+      <c r="H1" s="81"/>
+      <c r="I1" s="81"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="81"/>
+      <c r="O1" s="81"/>
+      <c r="P1" s="81"/>
+      <c r="Q1" s="81"/>
+      <c r="R1" s="81"/>
+      <c r="S1" s="81"/>
+      <c r="T1" s="81"/>
+      <c r="U1" s="81"/>
+      <c r="V1" s="81"/>
+      <c r="W1" s="81"/>
+      <c r="X1" s="81"/>
     </row>
     <row r="2" spans="1:24" ht="22" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -3135,7 +3138,7 @@
       <c r="H20" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I20" s="80" t="s">
+      <c r="I20" s="77" t="s">
         <v>449</v>
       </c>
       <c r="J20" s="10"/>
@@ -3181,7 +3184,7 @@
       <c r="H21" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I21" s="80" t="s">
+      <c r="I21" s="77" t="s">
         <v>449</v>
       </c>
       <c r="J21" s="10"/>
@@ -3233,7 +3236,7 @@
       <c r="H22" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I22" s="80" t="s">
+      <c r="I22" s="77" t="s">
         <v>449</v>
       </c>
       <c r="J22" s="10"/>
@@ -3383,7 +3386,7 @@
       <c r="H25" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I25" s="80" t="s">
+      <c r="I25" s="77" t="s">
         <v>449</v>
       </c>
       <c r="J25" s="10"/>
@@ -3617,7 +3620,7 @@
       <c r="H30" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I30" s="80" t="s">
+      <c r="I30" s="77" t="s">
         <v>444</v>
       </c>
       <c r="J30" s="10"/>
@@ -3663,7 +3666,7 @@
       <c r="H31" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I31" s="82" t="s">
+      <c r="I31" s="79" t="s">
         <v>447</v>
       </c>
       <c r="J31" s="10"/>
@@ -3755,7 +3758,7 @@
       <c r="H33" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I33" s="82" t="s">
+      <c r="I33" s="79" t="s">
         <v>443</v>
       </c>
       <c r="J33" s="10"/>
@@ -3939,7 +3942,7 @@
       <c r="H37" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I37" s="80" t="s">
+      <c r="I37" s="77" t="s">
         <v>446</v>
       </c>
       <c r="J37" s="10"/>
@@ -4081,7 +4084,7 @@
       <c r="H40" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I40" s="80" t="s">
+      <c r="I40" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J40" s="10"/>
@@ -4129,7 +4132,7 @@
       <c r="H41" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I41" s="82" t="s">
+      <c r="I41" s="79" t="s">
         <v>445</v>
       </c>
       <c r="J41" s="10"/>
@@ -4177,7 +4180,7 @@
       <c r="H42" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I42" s="80" t="s">
+      <c r="I42" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J42" s="10"/>
@@ -4223,7 +4226,7 @@
       <c r="H43" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I43" s="82" t="s">
+      <c r="I43" s="79" t="s">
         <v>445</v>
       </c>
       <c r="J43" s="10"/>
@@ -4269,7 +4272,7 @@
       <c r="H44" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I44" s="80" t="s">
+      <c r="I44" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J44" s="10"/>
@@ -4317,7 +4320,7 @@
       <c r="H45" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I45" s="80" t="s">
+      <c r="I45" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J45" s="10"/>
@@ -4367,7 +4370,7 @@
       <c r="H46" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I46" s="80" t="s">
+      <c r="I46" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J46" s="10"/>
@@ -4413,7 +4416,7 @@
       <c r="H47" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I47" s="80" t="s">
+      <c r="I47" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J47" s="10"/>
@@ -4459,7 +4462,7 @@
       <c r="H48" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I48" s="80" t="s">
+      <c r="I48" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J48" s="10"/>
@@ -4505,7 +4508,7 @@
       <c r="H49" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I49" s="80" t="s">
+      <c r="I49" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J49" s="10"/>
@@ -4551,7 +4554,7 @@
       <c r="H50" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I50" s="80" t="s">
+      <c r="I50" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J50" s="10"/>
@@ -4597,7 +4600,7 @@
       <c r="H51" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I51" s="80" t="s">
+      <c r="I51" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J51" s="10"/>
@@ -4643,7 +4646,7 @@
       <c r="H52" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I52" s="80" t="s">
+      <c r="I52" s="77" t="s">
         <v>445</v>
       </c>
       <c r="J52" s="10"/>
@@ -4739,7 +4742,7 @@
       <c r="H54" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I54" s="80" t="s">
+      <c r="I54" s="77" t="s">
         <v>446</v>
       </c>
       <c r="J54" s="10"/>
@@ -4785,7 +4788,7 @@
       <c r="H55" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I55" s="80" t="s">
+      <c r="I55" s="77" t="s">
         <v>446</v>
       </c>
       <c r="J55" s="10"/>
@@ -4831,7 +4834,7 @@
       <c r="H56" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I56" s="80" t="s">
+      <c r="I56" s="77" t="s">
         <v>446</v>
       </c>
       <c r="J56" s="10"/>
@@ -4879,7 +4882,7 @@
       <c r="H57" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I57" s="80" t="s">
+      <c r="I57" s="77" t="s">
         <v>448</v>
       </c>
       <c r="J57" s="10"/>
@@ -4925,7 +4928,7 @@
       <c r="H58" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I58" s="80" t="s">
+      <c r="I58" s="77" t="s">
         <v>446</v>
       </c>
       <c r="J58" s="10"/>
@@ -4971,7 +4974,7 @@
       <c r="H59" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I59" s="82" t="s">
+      <c r="I59" s="79" t="s">
         <v>444</v>
       </c>
       <c r="J59" s="10"/>
@@ -5017,7 +5020,7 @@
       <c r="H60" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I60" s="80" t="s">
+      <c r="I60" s="77" t="s">
         <v>444</v>
       </c>
       <c r="J60" s="10"/>
@@ -5063,7 +5066,7 @@
       <c r="H61" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I61" s="82" t="s">
+      <c r="I61" s="79" t="s">
         <v>444</v>
       </c>
       <c r="J61" s="10"/>
@@ -5109,7 +5112,7 @@
       <c r="H62" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I62" s="80" t="s">
+      <c r="I62" s="77" t="s">
         <v>444</v>
       </c>
       <c r="J62" s="10"/>
@@ -5477,7 +5480,7 @@
       <c r="H70" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I70" s="81" t="s">
+      <c r="I70" s="78" t="s">
         <v>28</v>
       </c>
       <c r="J70" s="10"/>
@@ -5529,7 +5532,7 @@
       <c r="H71" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I71" s="80" t="s">
+      <c r="I71" s="77" t="s">
         <v>442</v>
       </c>
       <c r="J71" s="10"/>
@@ -5903,7 +5906,7 @@
       <c r="H79" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I79" s="80" t="s">
+      <c r="I79" s="77" t="s">
         <v>443</v>
       </c>
       <c r="J79" s="10"/>
@@ -5951,7 +5954,7 @@
       <c r="H80" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I80" s="80" t="s">
+      <c r="I80" s="77" t="s">
         <v>443</v>
       </c>
       <c r="J80" s="10"/>
@@ -5999,7 +6002,7 @@
       <c r="H81" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I81" s="80" t="s">
+      <c r="I81" s="77" t="s">
         <v>443</v>
       </c>
       <c r="J81" s="10"/>
@@ -6047,7 +6050,7 @@
       <c r="H82" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I82" s="82" t="s">
+      <c r="I82" s="79" t="s">
         <v>48</v>
       </c>
       <c r="J82" s="10"/>
@@ -6481,6 +6484,35 @@
         <v>29</v>
       </c>
       <c r="X91" s="10"/>
+    </row>
+    <row r="92" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>90</v>
+      </c>
+      <c r="B92" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C92" t="s">
+        <v>450</v>
+      </c>
+      <c r="D92" s="13">
+        <v>46185</v>
+      </c>
+      <c r="E92" s="13">
+        <v>46186</v>
+      </c>
+      <c r="F92">
+        <v>2</v>
+      </c>
+      <c r="G92">
+        <v>88</v>
+      </c>
+      <c r="H92" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="I92" t="s">
+        <v>28</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:I91" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -6503,12 +6535,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="82" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
     </row>
     <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="54" t="s">
@@ -7091,12 +7123,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="82" t="s">
         <v>333</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
+      <c r="D1" s="81"/>
     </row>
     <row r="2" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="54" t="s">
@@ -7369,11 +7401,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="82" t="s">
         <v>388</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
+      <c r="B1" s="81"/>
+      <c r="C1" s="81"/>
     </row>
     <row r="2" spans="1:3" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="54" t="s">

</xml_diff>